<commit_message>
feat: plantilla en blanco con todos los campos del producto
- plantilla-productos-tiketes.xlsx: sin filas de ejemplo (en blanco) y con
  todos los campos de la pantalla de nuevo producto: nombre, precio, costo,
  stock, stock_minimo, categoria, unidad, marca, codigo_barras, sku,
  descripcion (la foto va en la app, no cabe en Excel).
- plantilla.html: documenta los 11 campos, aclara que solo nombre y precio son
  obligatorios, y que un Excel propio también sirve (la app lee por nombre de
  columna e ignora las que no reconoce).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantilla-productos-tiketes.xlsx
+++ b/plantilla-productos-tiketes.xlsx
@@ -466,14 +466,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -489,141 +495,49 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>costo</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>stock_minimo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>marca</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>codigo_barras</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>sku</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Coca Cola 600ml</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C2" t="n">
-        <v>50</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>bebidas</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>7501055310302</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Sabritas Clásicas 45g</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>16</v>
-      </c>
-      <c r="C3" t="n">
-        <v>80</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>snacks</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>7501011100015</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Galletas Marías 170g</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>18</v>
-      </c>
-      <c r="C4" t="n">
-        <v>40</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>galletas</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Leche Lala 1L</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>28</v>
-      </c>
-      <c r="C5" t="n">
-        <v>25</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>lacteos</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Pan Bimbo Integral</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>52</v>
-      </c>
-      <c r="C6" t="n">
-        <v>15</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>panaderia</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Jabón Roma 250g</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>14</v>
-      </c>
-      <c r="C7" t="n">
-        <v>60</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>limpieza</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>descripcion</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -636,11 +550,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -663,7 +577,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Obligatorio. Nombre del producto (máximo 100 caracteres).</t>
+          <t>OBLIGATORIO. Nombre del producto (máx. 100 caracteres).</t>
         </is>
       </c>
     </row>
@@ -675,151 +589,139 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Obligatorio. Precio de venta, mayor a 0. Usa punto o coma: 20 o 20.50</t>
+          <t>OBLIGATORIO. Precio de venta, mayor a 0. Ej: 20 o 20.50</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>stock</t>
+          <t>costo</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Cantidad en existencia. Número entero, 0 o más. Si lo dejas vacío, entra como 0.</t>
+          <t>Opcional. Lo que te cuesta a ti (para calcular ganancia).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>categoria</t>
+          <t>stock</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Una de la lista de abajo. Si no coincide, entra como "otros".</t>
+          <t>Opcional. Piezas en existencia. Entero, 0 o más. Vacío = 0.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>sku</t>
+          <t>stock_minimo</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Opcional. El código de barras del producto. Déjalo vacío si no lo tienes.</t>
+          <t>Opcional. Cuándo avisarte que ya casi se acaba. Entero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Opcional. Una de la lista de abajo. Si no coincide, entra como "otros".</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Categorías</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Escribe exactamente una de estas (en minúsculas):</t>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Opcional. pza, kg, lt, caja, etc. Vacío = pza.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>•</t>
+          <t>marca</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>abarrotes</t>
+          <t>Opcional. Marca del producto.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>•</t>
+          <t>codigo_barras</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>bebidas</t>
+          <t>Opcional. El código de barras. Si lo dejas vacío, lo escaneas después en la app.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>•</t>
+          <t>sku</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>lacteos</t>
+          <t>Opcional. Tu clave interna. Si lo dejas vacío, usa el código de barras.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>•</t>
+          <t>descripcion</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>snacks</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>panaderia</t>
+          <t>Opcional. Nota o detalle del producto.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>dulces</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>limpieza</t>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Deja los nombres de las columnas TAL CUAL. Solo "nombre" y "precio" son obligatorios; lo demás puedes dejarlo vacío.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>cuidado</t>
+          <t>Categorías</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Escribe exactamente una de estas (en minúsculas):</t>
         </is>
       </c>
     </row>
@@ -831,7 +733,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>mascotas</t>
+          <t>abarrotes</t>
         </is>
       </c>
     </row>
@@ -843,7 +745,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>galletas</t>
+          <t>bebidas</t>
         </is>
       </c>
     </row>
@@ -855,7 +757,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>papas</t>
+          <t>lacteos</t>
         </is>
       </c>
     </row>
@@ -867,89 +769,185 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>otros</t>
+          <t>snacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>panaderia</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Límites</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>Cuántos productos puedes tener según tu plan:</t>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>dulces</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>•</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>50 productos</t>
+          <t>limpieza</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Essential</t>
+          <t>•</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>500 productos</t>
+          <t>cuidado</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Pro</t>
+          <t>•</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>2,500 productos</t>
+          <t>mascotas</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>•</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>25,000 productos</t>
+          <t>galletas</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>papas</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>otros</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Límites</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Cuántos productos puedes tener según tu plan:</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>50 productos</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>500 productos</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>2,500 productos</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>25,000 productos</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
           <t>Fotos</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Las fotos no caben en el Excel: primero sube tus productos con este archivo (rápido, sin escanear uno por uno) y luego, en la app, agrega la foto a los productos que quieras. Los demás muestran la inicial de su nombre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>No caben en el Excel: sube primero tus productos con este archivo y luego, en la app, agrega la foto a los que quieras.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Importar</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>En la app: Productos → Importar → elige este archivo.</t>
         </is>

</xml_diff>